<commit_message>
Clean up project layout: drop bundled interpreter and old scripts, add UDT/Modbus tools
- Bundled CPython 3.13 removed from the folder (was untracked; now using system Python 3.14 via the py launcher).

- Removed superseded top-level scripts (Excel to Json*, Get Tag Names, extract_udt_tags, Ignition_UDT_Creation).

- Added UDT_Creation/ (ignition_udt_tool) and Device Configuration/ (CreateModbusDeviceFile) tools plus their Excel/JSON files.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/UDT_Creation_Test.xlsx
+++ b/UDT_Creation_Test.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\austin.funken\Documents\Projects\Python\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9A35E8B2-9836-4E5B-905A-FFACB993F046}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AAFCE5A-0AEF-4F3F-AB10-33091C989614}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{0E37F75F-5C54-435B-8C4E-8F6912250735}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{0E37F75F-5C54-435B-8C4E-8F6912250735}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="26">
   <si>
     <t>name</t>
   </si>
@@ -108,6 +108,12 @@
   </si>
   <si>
     <t>false|true</t>
+  </si>
+  <si>
+    <t>opcItemPath</t>
+  </si>
+  <si>
+    <t>ns=1;s=[{Device}]HR1</t>
   </si>
 </sst>
 </file>
@@ -479,7 +485,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0BA3DE22-C944-4BB9-B6C3-43931EF24461}">
-  <dimension ref="A1:N2"/>
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6" bestFit="1" customWidth="1"/>
@@ -487,18 +493,19 @@
     <col min="3" max="3" width="14.5703125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="7.7109375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="11.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="7.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17.7109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="22.42578125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="15.85546875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="7.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="17.7109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="22.42578125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="11" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="11.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -515,34 +522,37 @@
         <v>4</v>
       </c>
       <c r="F1" t="s">
+        <v>24</v>
+      </c>
+      <c r="G1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="M1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="N1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="O1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>14</v>
       </c>
@@ -556,30 +566,33 @@
         <v>17</v>
       </c>
       <c r="F2" t="s">
+        <v>25</v>
+      </c>
+      <c r="G2" t="s">
         <v>18</v>
       </c>
-      <c r="G2" t="s">
+      <c r="H2" t="s">
         <v>19</v>
       </c>
-      <c r="H2" t="s">
+      <c r="I2" t="s">
         <v>20</v>
       </c>
-      <c r="I2" t="b">
+      <c r="J2" t="b">
         <v>1</v>
       </c>
-      <c r="J2">
+      <c r="K2">
         <v>5</v>
       </c>
-      <c r="K2" t="s">
+      <c r="L2" t="s">
         <v>21</v>
       </c>
-      <c r="L2" t="s">
+      <c r="M2" t="s">
         <v>16</v>
       </c>
-      <c r="M2" t="s">
+      <c r="N2" t="s">
         <v>22</v>
       </c>
-      <c r="N2" t="s">
+      <c r="O2" t="s">
         <v>23</v>
       </c>
     </row>

</xml_diff>